<commit_message>
4/2 sửa lỗi bên quản lý điểm
</commit_message>
<xml_diff>
--- a/kma_mm/kma_be/src/exports/excel/danh_sach_cuoi_ky.xlsx
+++ b/kma_mm/kma_be/src/exports/excel/danh_sach_cuoi_ky.xlsx
@@ -85,6 +85,24 @@
     <t>1</t>
   </si>
   <si>
+    <t>test0101</t>
+  </si>
+  <si>
+    <t>Nguyễn Văn</t>
+  </si>
+  <si>
+    <t>Hòa</t>
+  </si>
+  <si>
+    <t>test01</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
     <t>test0102</t>
   </si>
   <si>
@@ -94,13 +112,7 @@
     <t>Bình</t>
   </si>
   <si>
-    <t>test01</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>2</t>
+    <t>3</t>
   </si>
   <si>
     <t>test0103</t>
@@ -112,7 +124,7 @@
     <t>Cường</t>
   </si>
   <si>
-    <t>3</t>
+    <t>4</t>
   </si>
   <si>
     <t>test0104</t>
@@ -124,21 +136,21 @@
     <t>Dũng</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>test0101</t>
-  </si>
-  <si>
-    <t>Nguyễn Văn</t>
-  </si>
-  <si>
-    <t>Hòa</t>
-  </si>
-  <si>
     <t>5</t>
   </si>
   <si>
+    <t>test0105</t>
+  </si>
+  <si>
+    <t>Vũ</t>
+  </si>
+  <si>
+    <t>Hưng</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
     <t>test0106</t>
   </si>
   <si>
@@ -146,18 +158,6 @@
   </si>
   <si>
     <t>Huy</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>test0105</t>
-  </si>
-  <si>
-    <t>Vũ</t>
-  </si>
-  <si>
-    <t>Hưng</t>
   </si>
   <si>
     <t>Hà Nội, ngày ___ tháng ___ năm 20___</t>
@@ -684,7 +684,7 @@
     <col min="2" max="2" width="5.28" customWidth="1"/>
     <col min="3" max="3" width="13.799999999999999" customWidth="1"/>
     <col min="4" max="4" width="22.548" customWidth="1"/>
-    <col min="5" max="5" width="9.096" customWidth="1"/>
+    <col min="5" max="5" width="16.296" customWidth="1"/>
     <col min="6" max="6" width="9.251999999999999" customWidth="1"/>
     <col min="7" max="7" width="7.548" customWidth="1"/>
     <col min="8" max="8" width="9.251999999999999" customWidth="1"/>
@@ -867,7 +867,7 @@
         <v>27</v>
       </c>
       <c r="H12" s="6">
-        <v>4.7</v>
+        <v>0.9</v>
       </c>
       <c r="I12" s="6" t="s">
         <v>27</v>
@@ -899,7 +899,7 @@
         <v>27</v>
       </c>
       <c r="H13" s="8">
-        <v>7.3</v>
+        <v>4.4</v>
       </c>
       <c r="I13" s="8" t="s">
         <v>27</v>
@@ -931,7 +931,7 @@
         <v>27</v>
       </c>
       <c r="H14" s="8">
-        <v>7</v>
+        <v>7.3</v>
       </c>
       <c r="I14" s="8" t="s">
         <v>27</v>
@@ -963,7 +963,7 @@
         <v>27</v>
       </c>
       <c r="H15" s="8">
-        <v>4.5</v>
+        <v>7</v>
       </c>
       <c r="I15" s="8" t="s">
         <v>27</v>
@@ -995,7 +995,7 @@
         <v>27</v>
       </c>
       <c r="H16" s="8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I16" s="8" t="s">
         <v>27</v>
@@ -1027,7 +1027,7 @@
         <v>27</v>
       </c>
       <c r="H17" s="10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I17" s="10" t="s">
         <v>27</v>
@@ -1088,7 +1088,7 @@
     <mergeCell ref="G20:J20"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.4" right="0.4" top="0.2" bottom="0.2" header="0.3" footer="0.3"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.2" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
</xml_diff>